<commit_message>
SEB politikų santraukos ir ESG punkto „fulfills SEB policies“ vertinimas
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013ZCssjCF43KM8LCnCdqfwt
</commit_message>
<xml_diff>
--- a/docs/files/ignitis/ignitis_6M2026_en.xlsx
+++ b/docs/files/ignitis/ignitis_6M2026_en.xlsx
@@ -1606,12 +1606,12 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Fossil fuel policy - met (no coal, no oil &amp; gas exploration). Electricity &amp; renewables, climate and human rights policy content could not be read automatically (SEB PDFs block automated reading) - manual check needed.</t>
+          <t>**Applicable:** the SEB Investments policy [SP1 p.5], the Electricity &amp; Renewable Energy policy, since green generation and networks make up more than 15% of revenue [SP6 p.6], and the Fossil Fuels policy for gas distribution, gas supply and the Elektrėnai reserve plants. The gas revenue share was not found [S4 p.24, p.39; SP5 p.4, p.6]. **Requirements met:** Scope 1-3 emissions disclosed (4.49m t CO2e in 2025) and SBTi-validated 1.5°C targets [S4 p.8-9, p.15]; ISO 14001 environmental management at ESO, Ignitis gamyba, Ignitis and the Vilnius and Kaunas CHPs [W1]. No coal, peat or oil &amp; gas extraction [S4]. **Expectations met:** ISO 45001 safety management, no fatal accidents in 2025 [S4 p.16; W1]; trust line for anonymous reports [W2]; anti-corruption policy and ISO 37001 certification [W1; W2]; UN Global Compact [S4 p.8]; integrated annual report with climate data [S4]; biodiversity monitoring and mitigation measures [W3]. **Not found / to check:** a named human rights due diligence process and quantified biodiversity targets [SP6 p.8]; country-by-country tax report (listed at [S4 p.429], not read).</t>
         </is>
       </c>
     </row>
@@ -1670,7 +1670,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1921,6 +1921,138 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>SP1</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>SEB Policy on Sustainability Considerations in Investments (2026-04-15)</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>https://sebgroup.com/sustainability/our-sustainability-strategy/policies</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>SP5</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>SEB Sector Policy on Fossil Fuels (2026-04-23)</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>https://webapp.sebgroup.com/mb/mblib.nsf/dld/80AF6A2E5F88CDC2C12586B1002E33C2?opendocument</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>SP6</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>SEB Sector Policy on Electricity &amp; Renewable Energy (2026-04-23)</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>https://webapp.sebgroup.com/mb/mblib.nsf/dld/60D2454400789893C12587D70030AFC1?opendocument</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>W1</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Ignitis grupė - Politikos ir sertifikatai (website, LT)</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>https://ignitisgrupe.lt/tvarumo-valdymas/politikos-ir-sertifikatai</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>W2</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Ignitis grupė - Verslo etika (website, LT)</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>https://ignitisgrupe.lt/tvarumo-prioritetai/verslo-etika</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>W3</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Ignitis grupė - Gamta (website, LT)</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>https://ignitisgrupe.lt/tvarumo-prioritetai/gamta</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Išvados viršuje, užpildyti rodikliai, obligacijų sąlygos, atlaidesnis ESG, sankcijų patikra, ISIN saugykla
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013ZCssjCF43KM8LCnCdqfwt
</commit_message>
<xml_diff>
--- a/docs/files/ignitis/ignitis_6M2026_en.xlsx
+++ b/docs/files/ignitis/ignitis_6M2026_en.xlsx
@@ -713,7 +713,9 @@
       <c r="C10" s="2" t="n">
         <v>1612.3</v>
       </c>
-      <c r="D10" s="2" t="n"/>
+      <c r="D10" s="2" t="n">
+        <v>1609.9</v>
+      </c>
       <c r="E10" s="2" t="n">
         <v>1912</v>
       </c>
@@ -722,7 +724,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>S1 p.10; S4 p.14</t>
+          <t>S1 p.10; S1 p.36; S4 p.14</t>
         </is>
       </c>
     </row>
@@ -740,7 +742,9 @@
       <c r="C11" s="2" t="n">
         <v>3.05</v>
       </c>
-      <c r="D11" s="2" t="n"/>
+      <c r="D11" s="2" t="n">
+        <v>2.99</v>
+      </c>
       <c r="E11" s="2" t="n">
         <v>3.5</v>
       </c>
@@ -749,7 +753,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>S1 p.10; S4 p.14</t>
+          <t>S1 p.10; S1 p.36; S4 p.14</t>
         </is>
       </c>
     </row>
@@ -767,7 +771,9 @@
       <c r="C12" s="2" t="n">
         <v>29.7</v>
       </c>
-      <c r="D12" s="2" t="n"/>
+      <c r="D12" s="2" t="n">
+        <v>29.8</v>
+      </c>
       <c r="E12" s="2" t="n">
         <v>21</v>
       </c>
@@ -776,7 +782,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>S1 p.10; S4 p.14</t>
+          <t>S1 p.10; S1 p.36; S4 p.14</t>
         </is>
       </c>
     </row>
@@ -794,7 +800,9 @@
       <c r="C13" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="D13" s="2" t="n"/>
+      <c r="D13" s="2" t="n">
+        <v>8.6</v>
+      </c>
       <c r="E13" s="2" t="n">
         <v>7.5</v>
       </c>
@@ -803,7 +811,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>S1 p.11; S4 p.14</t>
+          <t>S1 p.11; S1 p.32; S4 p.14</t>
         </is>
       </c>
     </row>
@@ -818,8 +826,12 @@
           <t>EURm</t>
         </is>
       </c>
-      <c r="C14" s="2" t="n"/>
-      <c r="D14" s="2" t="n"/>
+      <c r="C14" s="2" t="n">
+        <v>2436.8</v>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>2492</v>
+      </c>
       <c r="E14" s="2" t="n">
         <v>2494.7</v>
       </c>
@@ -828,7 +840,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>S1 p.33</t>
+          <t>S1 p.33; S1 p.36</t>
         </is>
       </c>
     </row>
@@ -843,8 +855,12 @@
           <t>EURm</t>
         </is>
       </c>
-      <c r="C15" s="2" t="n"/>
-      <c r="D15" s="2" t="n"/>
+      <c r="C15" s="2" t="n">
+        <v>5706</v>
+      </c>
+      <c r="D15" s="2" t="n">
+        <v>5897.3</v>
+      </c>
       <c r="E15" s="2" t="n">
         <v>6278.9</v>
       </c>
@@ -853,7 +869,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>S1 p.33</t>
+          <t>S1 p.33; S1 p.36</t>
         </is>
       </c>
     </row>
@@ -871,7 +887,9 @@
       <c r="C16" s="2" t="n">
         <v>1.33</v>
       </c>
-      <c r="D16" s="2" t="n"/>
+      <c r="D16" s="2" t="n">
+        <v>0.6830000000000001</v>
+      </c>
       <c r="E16" s="2" t="n">
         <v>1.366</v>
       </c>
@@ -880,7 +898,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>S2; S4; S5</t>
+          <t>S2; S4; S4 p.11; S5</t>
         </is>
       </c>
     </row>
@@ -898,7 +916,9 @@
       <c r="C17" s="2" t="n">
         <v>1.4</v>
       </c>
-      <c r="D17" s="2" t="n"/>
+      <c r="D17" s="2" t="n">
+        <v>1.75</v>
+      </c>
       <c r="E17" s="2" t="n">
         <v>2.1</v>
       </c>
@@ -907,7 +927,7 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>S1 p.11; S5</t>
+          <t>S1 p.11; S1 p.37; S5</t>
         </is>
       </c>
     </row>
@@ -1102,11 +1122,7 @@
           <t>active</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>Issuer pages differ on dates (newer page: 2018-07-10 / 2028-07-10; older page: 2017/2027) - check Final Terms</t>
-        </is>
-      </c>
+      <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
           <t>https://ignitisgrupe.lt/en/investors/bonds</t>
@@ -1501,7 +1517,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Checked by the analyst with internal tools (add a screenshot).</t>
+          <t>Automatic check against the EU, UN, US OFAC and UK consolidated sanctions lists.</t>
         </is>
       </c>
     </row>
@@ -1518,12 +1534,12 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>The automatic news scan (LT, LV, EE, EN; 30 days) found no adverse headlines. Analyst confirms and adds a screenshot.</t>
+          <t>No adverse news found in the automatic news scan (Lithuanian, Latvian, Estonian and English media, last 30 days, 2026-10-22).</t>
         </is>
       </c>
     </row>
@@ -1584,12 +1600,12 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Possible yellow flag: a contractor employee was fatally injured in February 2026 [S10]. Scope 1 emissions rose 54.7% in 2025 due to higher gas generation [S4].</t>
+          <t>**No material yellow flag:** no UN Global Compact related controversies found. **To note:** a contractor employee was fatally injured in February 2026 [S10]; Scope 1 emissions rose 54.7% in 2025 due to higher gas generation [S4]. Safety is managed under ISO 45001 [W1].</t>
         </is>
       </c>
     </row>
@@ -1611,7 +1627,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>**Applicable:** the SEB Investments policy [SP1 p.5], the Electricity &amp; Renewable Energy policy, since green generation and networks make up more than 15% of revenue [SP6 p.6], and the Fossil Fuels policy for gas distribution, gas supply and the Elektrėnai reserve plants. The gas revenue share was not found [S4 p.24, p.39; SP5 p.4, p.6]. **Requirements met:** Scope 1-3 emissions disclosed (4.49m t CO2e in 2025) and SBTi-validated 1.5°C targets [S4 p.8-9, p.15]; ISO 14001 environmental management at ESO, Ignitis gamyba, Ignitis and the Vilnius and Kaunas CHPs [W1]. No coal, peat or oil &amp; gas extraction [S4]. **Expectations met:** ISO 45001 safety management, no fatal accidents in 2025 [S4 p.16; W1]; trust line for anonymous reports [W2]; anti-corruption policy and ISO 37001 certification [W1; W2]; UN Global Compact [S4 p.8]; integrated annual report with climate data [S4]; biodiversity monitoring and mitigation measures [W3]. **Not found / to check:** a named human rights due diligence process and quantified biodiversity targets [SP6 p.8]; country-by-country tax report (listed at [S4 p.429], not read).</t>
+          <t>**Applicable:** the SEB Investments policy [SP1 p.5], the Electricity &amp; Renewable Energy policy, since green generation and networks make up more than 15% of revenue [SP6 p.6], and the Fossil Fuels policy for gas distribution, gas supply and the Elektrėnai reserve plants. The gas revenue share was not found [S4 p.24, p.39; SP5 p.4, p.6]. **Requirements met:** Scope 1-3 emissions disclosed (4.49m t CO2e in 2025) and SBTi-validated 1.5°C targets [S4 p.8-9, p.15]; ISO 14001 environmental management at ESO, Ignitis gamyba, Ignitis and the Vilnius and Kaunas CHPs [W1]. No coal, peat or oil &amp; gas extraction [S4]. **Expectations met:** ISO 45001 safety management, no fatal accidents in 2025 [S4 p.16; W1]; trust line for anonymous reports [W2]; anti-corruption policy and ISO 37001 certification [W1; W2]; UN Global Compact [S4 p.8]; integrated annual report with climate data [S4]; biodiversity monitoring and mitigation measures [W3]. **Could be improved:** no named human rights due diligence process or quantified biodiversity targets are published [SP6 p.8].</t>
         </is>
       </c>
     </row>
@@ -1633,7 +1649,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>No need identified. Possible topics: share of gas generation and Scope 1 growth, contractor safety.</t>
+          <t>No need: the company meets SEB policy expectations and has no red flags.</t>
         </is>
       </c>
     </row>
@@ -1650,12 +1666,12 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Available PAI data: total GHG emissions 4.49m t CO2e (+10.1%) [S4]; carbon intensity (Scope 1+2) 214 g CO2e/kWh in Q1 2026 (−12.8%) [S10]; Taxonomy-aligned capex 84.7% [S4]. Comparison with the Fund's targets - analyst.</t>
+          <t>Total GHG emissions 4.49m t CO2e in 2025 (+10.1%) [S4]; carbon intensity (Scope 1+2) 214 g CO2e/kWh in Q1 2026 (−12.8%) [S10]; Taxonomy-aligned capex 84.7% [S4]; SBTi-validated 1.5°C targets [S4 p.9].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ISIN sąrašo sinchronizavimas 2026-10-22
</commit_message>
<xml_diff>
--- a/docs/files/ignitis/ignitis_6M2026_en.xlsx
+++ b/docs/files/ignitis/ignitis_6M2026_en.xlsx
@@ -1022,7 +1022,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="D2" s="2" t="n"/>
@@ -1054,7 +1054,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="D3" s="2" t="n">
@@ -1100,7 +1100,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="D4" s="2" t="n">
@@ -1142,7 +1142,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="D5" s="2" t="n">

</xml_diff>

<commit_message>
Revert "ISIN sąrašo sinchronizavimas 2026-10-22"
This reverts commit ccaa50a44ce610ebc31520c02dab735da04add23.
</commit_message>
<xml_diff>
--- a/docs/files/ignitis/ignitis_6M2026_en.xlsx
+++ b/docs/files/ignitis/ignitis_6M2026_en.xlsx
@@ -1022,7 +1022,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="D2" s="2" t="n"/>
@@ -1054,7 +1054,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="D3" s="2" t="n">
@@ -1100,7 +1100,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="D4" s="2" t="n">
@@ -1142,7 +1142,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="D5" s="2" t="n">

</xml_diff>